<commit_message>
Updated store-scope authentication and all corresponding tests
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/order_archive/Webstaurant/Webstaurant_Triphammer_20260624.xlsx
+++ b/WorkBot/main/data/order_archive/Webstaurant/Webstaurant_Triphammer_20260624.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,43 +482,64 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>104APRICOT28</t>
+          <t>111QUINTRORG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Apricot - Dried</t>
+          <t>Quinoa - Tri Color</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>128.49</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>128.49</v>
+        <v>196.47</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>111QUINTRORG</t>
+          <t>3463306BK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Quinoa - Tri Color</t>
+          <t>Ladle - Black Plastic (2oz)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>65.48999999999999</v>
+        <v>21.33</v>
       </c>
       <c r="E7" t="n">
-        <v>196.47</v>
+        <v>21.33</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>128HD24COMBO</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Container - HD Deli soup (24oz) w/ Lid</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="E8" t="n">
+        <v>28.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>